<commit_message>
Update datasets with final iteration linguist verification
</commit_message>
<xml_diff>
--- a/Dataset/Test_Set.xlsx
+++ b/Dataset/Test_Set.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E162"/>
+  <dimension ref="A1:E123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,4347 +458,3294 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>anak sa sala</t>
+          <t>dula og panit</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>usa ka anak nga dili-konsejero</t>
+          <t>sa pag- masturba</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>['sala']</t>
+          <t>['dula']</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ang anak sa sala nga si Maria kay ginaatiman gihapon sa iyang lola ug lolo.</t>
+          <t>Si Maria nagbuot-buot kay gusto siya magdula og panit pirmi.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Ang anak sa sala nagdula duol sa altar samtang nagaampo ang pari.</t>
+          <t>Ang akong manghod nagdula og panit sa iyang baboy-baboy nga dulaan.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>gibuhi</t>
+          <t>murag gitilapan og iring</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ang penis sa usa ka lalaki</t>
+          <t>walay sapayan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>['gibuhi']</t>
+          <t>['gitilapan']</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ang mga bata nga iyang gibuhi kay nagdako nga maayong laki.</t>
+          <t>"Ang iyang mga gamit sa opisina murag gitilapan og iring, limpyo ug hapsay."</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Si Lola ang gibuhi sa among gidala nga gamay nga iro gikan sa dalan.</t>
+          <t>"Pagkakita nako sa lamisa, murag gitilapan og iring kay walay tanang bahaw nga niwangig."</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>nadakpan na ba ang nagtupi nimo</t>
+          <t>litik</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>gisultihan sa usa ka tawo nga adunay bag-ong buhok</t>
+          <t>sa pag-aghat sa tudlo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>['nagtupi']</t>
+          <t>['litik']</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Nadakpan na ba ang nagtupi nimo nga wala man nindot imong buhok?</t>
+          <t>Ang mga tawo nga naglitik sa ilang mga pangandoy kasagaran magmalampuson.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Gidala dayon siya sa istasyon sa pulis ug giingnan nga "Nadakpan na ba ang nagtupi nimo nga wala man mangayo og permiso?"</t>
+          <t>Naglingkod si Juan sa lamisa ug kalit niyang gilitik ang botelya nga nagbarog.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>buotan ra og matulog</t>
+          <t>gi-indian</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>malinong</t>
+          <t>sa tinuyo nga dili motuman sa usa ka appointment</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>['matulog']</t>
+          <t>['gi-indian']</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Si Pedro buotan ra og matulog, kay pirmi lang magbinuang sa klase.</t>
+          <t>Ang iyang kauban sa trabaho gi-indian siya sa ilang meeting.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Si Lola kung mahigda, buotan ra og matulog kay dili siya maglihok-lihok sa gabii.</t>
+          <t>Ang tribo nga among gi-adtoan sa bukid, gi-indian sa mga lumad.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>murag langaw nga nakatugdon sa kabaw</t>
+          <t>pangatulig luwag</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>nouveau riche</t>
+          <t>gigamit sa pag-undang sa usa ka tawo nga misquoted o misheard sa usa ka gisulti</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>['nakatugdon']</t>
+          <t>['pangatulig']</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>"Siya karon murag langaw nga nakatugdon sa kabaw, taas kaayo og pride."</t>
+          <t>"Ayaw pag pangatulig luwag, klaroha imong mga desisyon."</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Pag-adlaw, nakita nako ang langaw nga nakatugdon sa likod sa kabaw samtang nag-id-id kini ug mga sanga.</t>
+          <t>Nagpangatulig luwag ang bata tungod kay busog kaayo siya human mikaon og daghang lugaw.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>kang kinsa man na imong sala</t>
+          <t>hatod og patay</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>gigamit sa pagsulti sa usa ka tawo nga sila lamang ang may sala sa ilang kaugalingon alang sa ilang kaugalingong mga problema</t>
+          <t>sa pagtambong sa usa ka paglubong o seremonya sa paghinumdom</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>['sala']</t>
+          <t>['hatod', 'patay']</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Kang kinsa man na imong sala nga nagdako ka ug kalit?</t>
+          <t>Ang mga tawo nga hatod og patay kasagaran nagpakita ug respeto sa namatay.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>"Giimbestigahan sa konsehal ang panghitabo, ug nangutana siya kang kinsa man na imong sala nga nahitabo ang aksidente."</t>
+          <t>Ang drayber mihangyo nga tabangan siya sa paghatod og patay ngadto sa sementeryo.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ayaw adto og gubat kon wala kay bala</t>
+          <t>hunaw</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ayaw pagbuhat ug dili-andam</t>
+          <t>sa paghunaw sa kamot sa usa o sa uban</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>['ayaw', 'adto']</t>
+          <t>['hunaw']</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ang mga negosyante giingnan nga ayaw adto og gubat kon wala kay bala sa kompetisyon.</t>
+          <t>Ang iyang kauban naghunaw sa mga problema aron dili siya maapil.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ang mga sundalo giingnan sa ilang kumander, "Ayaw adto og gubat kon wala kay bala, kay delikado ang kahimtang diha."</t>
+          <t>Nagpareha sila paghuman sa trabaho ug naghunaw sa ilang kamot sa kusina aron limpyo.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>mag-ugbok og mohon</t>
+          <t>ul-ol</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>sa pagpakigsekso</t>
+          <t>sa pag- masturba Mga sinonim: batil</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>['mag-ugbok']</t>
+          <t>['ul-ol']</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Si Ana nagplano nga mag-ugbok og mohon sa iyang birthday.</t>
+          <t>Ang iyang buhat kay ul-ol kaayo, wala gyud maghunahuna.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ang mga trabahante mag-ugbok og mohon aron magtukod og bag-ong balay.</t>
+          <t>Migawas sa ilang klase, nag-ul-ol siya sa ilang balay alang sa pagkat-on sa leksyon.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>mingaw pa ang panagat</t>
+          <t>nadakpan na</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>oras sa adlaw nga ang usa ka establisimento adunay pipila ka kostumer ug dili kaayo busy</t>
+          <t>gisultihan sa usa ka tawo nga adunay bag-ong buhok</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['nadakpan']</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Ang mga negosyo kasagaran mingaw pa ang panagat sa mga sayong oras.</t>
+          <t>Nadakpan na si Pedro nga nagsige ug pangawat sa tindahan.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Ang mga manginisda nanguli na kay mingaw pa ang panagat tungod sa bagyo.</t>
+          <t>Nadakpan na ang kawatan nga nisulod sa balay gabii.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dili madala og rosaryo</t>
+          <t>paabang</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>usa ka hingpit nga walay paglaom nga kahimtang</t>
+          <t>pag-abang</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>['madala']</t>
+          <t>['paabang']</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Si Pedro nag-atubang sa mga pagsulay nga dili madala og rosaryo.</t>
+          <t>Ang mga kwartong ipaabang kay dali ra kaayo mahurot ug ma-book.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Nag-ingon ang pari nga ang problema sa kalibutan dili madala og rosaryo ug mga pag-ampo lang.</t>
+          <t>"Nagpaabang sila sa ilang balay samtang nagbakasyon."</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>higda sa lubi</t>
+          <t>gigukod sa sudlay</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>pag-ula</t>
+          <t>nga walay buhok</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>['higda']</t>
+          <t>['gigukod']</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi lang higda sa lubi kung mag-inom.</t>
+          <t>Si Ana pirmi lang gigukod sa sudlay, kay dili siya ganahan mag-comb sa iyang buhok.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Ang bata nagduwa sa baybayon ug kalit lang mihigda sa lubi nga napalid sa balas.</t>
+          <t>Si Maria naglupad-lupad ang buhok samtang gigukod sa sudlay sa iyang manghod.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>walay man kardaba mamunga og tundan</t>
+          <t>buhat ang pasulti-on dili sulti ang pabuhaton</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ang mansanas dili mahulog nga layo sa kahoy</t>
+          <t>Maglakaw sa paghisgot</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['pasulti-on, pabuhaton']</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ang mga estudyante giingnan nga walay man kardaba mamunga og tundan, mao nga magtuon sila pag-ayo.</t>
+          <t>Si Juan giingnan nga buhat ang pasulti-on dili sulti ang pabuhaton sa iyang trabaho.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ang akong lolo kanunay magsulti nga walay man kardaba mamunga og tundan, mao nga ang among mga punuan sa saging dris likod balay pulos gyud mga kardaba.</t>
+          <t>"Sa klase sa sining, gipahimo sa maestro ang mga estudyante ug kaugalingong mga proyekto aron buhat ang pasulti-on dili sulti ang pabuhaton."</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>bisan ang kabaw nga naay upat ka tiil masipyat</t>
+          <t>abot sa pikas bukid</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>kitang tanan magkamali</t>
+          <t>usa ka tawo nga naghisgot nga makusog</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>['naay', 'masipyat']</t>
+          <t>['abot']</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Si Maria nasipyat sa pagplano, bisan ang kabaw nga naay upat ka tiil masipyat.</t>
+          <t>Ang istorya ni Pedro abot sa pikas bukid bisan dili tinuod.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ang kabaw nga naay upat ka tiil masipyat sa pagtabok sa pilapila ug nakasulod kini sa umahan.</t>
+          <t>Naglakaw mi ug dugay hangtod nga among naabtan ang pikas bukid.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Chona Mae</t>
+          <t>miulbo ang kaspa</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tsunami!</t>
+          <t>sa pag-abli ngadto sa kasuko</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>['Chona']</t>
+          <t>['miulbo']</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Si Chona Mae pirmi lang magbinuang sa eskwelahan.</t>
+          <t>Si Ana miulbo ang kaspa human nabal-an nga gilimbongan siya.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Si Chona Mae akong silingan nga kanunay akong kaistorya matag buntag.</t>
+          <t>Human sa dugang duha ka adlaw nga walay ligo, si Pedro nakabantay nga miulbo ang kaspa sa iyang ulo.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>abli ang Gaisano</t>
+          <t>pangatulig luwag</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>nga ang usa nga mosul-ob</t>
+          <t>gigamit sa pag-undang sa usa ka tawo nga misquoted o misheard sa usa ka gisulti</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['pangatulig']</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Kung abli ang Gaisano, kinahanglan dayon sirad-an aron dili magkatawa ang uban.</t>
+          <t>"Pangatulig luwag kaayo imong mga istorya, walay klaro."</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>"Dali na ta kay abli ang Gaisano ug daghan kaayong baligya nga barato."</t>
+          <t>Sa pagkahuman sa panihapon, gikuha ni Lola ang pangatulig luwag aron masimhot ang baho sa nilung-ag nga mais.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>batang murag korek</t>
+          <t>dili na mabalik ang baha paingon sa bukid</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>dili-matag-as</t>
+          <t>Ang nahimo dili mahimong malikayan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>['batang']</t>
+          <t>['mabalik']</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Ang batang murag korek nga si Lito pirmi lang nagbuot-buot.</t>
+          <t>Ang mga estudyante nakabalo nga dili na mabalik ang baha paingon sa bukid, mao nga nagplano na sila pag-ayo.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ang batang nagdula sa balas falor murag korek kay tan-aw nimo layo ra siya sa uban.</t>
+          <t>Pagkahuman sa kusog nga ulan, ang mga taga-barangay nag-istorya nga bisan unsaon pa, dili na mabalik ang baha paingon sa bukid, kay daghan kaayo ang tubig nga midiretso sa dagat.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>magpalapad og papel</t>
+          <t>manira sa dalan</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>aron magbaton ug dungog sa buhat sa uban</t>
+          <t>aron magpabilin nga magmata hangtod sa gabii</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>['magpalapad']</t>
+          <t>['manira']</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Ang mga tawo nga magpalapad og papel kasagaran dili tinood nga maayong magtrabaho.</t>
+          <t>"Ayaw pag manira sa dalan, klaroha imong mga desisyon."</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ang mga bata sa klase nagpalapad og papel gamit ang pintal para sa ilang proyekto sa arte.</t>
+          <t>"Ang negosyante manira sa dalan aron duna sila'y halin bisan sa gabii."</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>lunod patay</t>
+          <t>gilawog sa tirong</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>dihard</t>
+          <t>sa pagbutang sa peligro sa usa ka tawo, ilabina</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>['lunod', 'patay']</t>
+          <t>['gilawog']</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Si Pedro lunod patay sa iyang prinsipyo, dili gyud magbag-o.</t>
+          <t>Si Juan gilawog sa tirong, bisan wala siya naghimo sa sayop.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Ang biktima nakit-an nga lunod patay sa dagat human sa kusog nga bagyo.</t>
+          <t>Ang ilaga gilawog sa tirong aron kini dali madakop.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>hinaw</t>
+          <t>murag namatyag iring</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>sa paghunaw sa kamot sa usa o sa uban</t>
+          <t>gigamit sa paghulagway sa usa ka tawo nga nagtangis nga nagtangis o nagtangis nga nagtangis</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>['hinaw']</t>
+          <t>['namatyag']</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Ang iyang kauban naghinaw sa problema kay dili siya gusto maapil.</t>
+          <t>"Ang bata murag namatyag iring, hilak kaayo pagnalaya."</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>"Naghugaw ang iyang mga kamot sa pintal busa siya mihunaw dayon sa gripo."</t>
+          <t>Ang iring sa atop murag namatyag iring, kusog kaayo ang pangubog.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>kusog mokaon og gasolina</t>
+          <t>manglutasay</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>gas-gussing</t>
+          <t>usa ka manunulak sa mga bukog</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>['mokaon']</t>
+          <t>['manglutasay']</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Ang mga tawo nga mag-drive ug sakyanan nga kusog mokaon og gasolina kasagaran maglisod sa gasto.</t>
+          <t>Ang iyang kauban sa trabaho manglutasay sa mga kabataan.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Ang makina sa among sakyanan kusog mokaon og gasolina kung nagdagan mi sa highway.</t>
+          <t>Ang mga bata nagdula sa ilalom sa manglutasay aron magpa-uyog.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>dula og panit</t>
+          <t>habwa ang kinaon</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>sa pag- masturba</t>
+          <t>pag-awhag</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>['dula']</t>
+          <t>['habwa', 'kinaon']</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Ang iyang barkada kay dula og panit, bisan unsa na lang nga kalipay ang gihimo.</t>
+          <t>Si Maria naghabwa ang kinaon kay nagkalibanga.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Ang bata nagdula og panit sa daplin sa suba, gamit ang tanom nga iya nakuha gikan sa palibot.</t>
+          <t>Naghabwa ang bata sa kinaon gikan sa basket aron ipakaon sa mga iro.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>makagisi og pitaka</t>
+          <t>gadalag ulan</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>mahal kaayo</t>
+          <t>usa ka lalaki nga homoseksual</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['nagdala']</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Si Maria nakapalit ug bag nga makagisi og pitaka tungod sa kamahal.</t>
+          <t>Ang mga tawo nga gadalag ulan kasagaran naglisod sa pagdawat sa uban.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Ang kawatan nakagisi og pitaka aron makuha ang sulod niining kwarta.</t>
+          <t>Ang itom nga panganod sa langit gadalag ulan nga kusog kaayo.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>makamala og sapa</t>
+          <t>kuskos-balungos</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ang usa ka tawo nga may dagkong tiil</t>
+          <t>alternatibong pagsulat sa kuskos balungos</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>['makamala']</t>
+          <t>['kuskos']</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Si Pedro makamala og sapa kay grabe kaayo kadako ang tiil.</t>
+          <t>Si Ana pirmi lang kuskos-balungos kung naay buhaton nga dili siya ganahan.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Ang babaye makamala og sapa kay nahanaw ang tulay.</t>
+          <t>Gikuha ni Maria ang kutsilyo ug gigamit kini alang sa kuskos-balungos sa kinay sa isda.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>binatilay</t>
+          <t>taliba</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>sa pag-aghat sa usag usa sa mga penis</t>
+          <t>ang mga genital sa babaye</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>['binatilay']</t>
+          <t>['taliba']</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Ang mga batan-on nga nagdula og binatilay sa eskwelahan kay gipahimangnoan sa mga maestro.</t>
+          <t>Ang mga guwardiya nag-taliba sa building adlaw ug gabii.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Nagpasabot ang tigulang nga ang binatilay sa una kay bahin sa ilang tradisyonal nga sayaw nga gihimo panahon sa pista.</t>
+          <t>Ang taliba sa eskuylahan nagreport nga walay kakulian ang mga estudyante karong adlawa.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sabong</t>
+          <t>manakop og ligid</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>usa ka kompetisyon</t>
+          <t>nga ang usa ka tawo naugtang sa usa ka sakyanan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>['sabong']</t>
+          <t>['manakop']</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Ang mga sabong sa probinsya kasagaran ginadumog sa mga lokal nga residente.</t>
+          <t>Si Pedro manakop og ligid kay nagdagan-dagan sa kalsada.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>"Ang sabong nga gigamit nako sa pagpaligo humot ug daghan ug sabon."</t>
+          <t>Nagdula mi og dakop-dakop sa plaza unya nakalingkod ko para mopahuway, apan kalit nga miingon ang akong amigo nga manakop og ligid mi sa mga sakyanan nga nag-agi atubangan sa balay.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>lunod patay</t>
+          <t>buhat ang pasulti-on dili sulti ang pabuhaton</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>dihard</t>
+          <t>Maglakaw sa paghisgot</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>['lunod', 'patay']</t>
+          <t>['pasulti-on, pabuhaton']</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Ang iyang amigo lunod patay sa iyang pagtuo bisan pa sa mga pagsulay.</t>
+          <t>Ang mga tawo nga buhat ang pasulti-on dili sulti ang pabuhaton kasagaran magmalampuson.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Ang sakayan ilang gisakyan nasangit sa dagkong balod, ug nahinumdom ko sa babaye nga lunod patay sa ubos sa dagat.</t>
+          <t>Si Mario ang nagtrabaho sa proyekto, mao nga buhat ang pasulti-on dili sulti ang pabuhaton aron klaro ang panabang.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>murag langaw nga nakatugdon sa kabaw</t>
+          <t>lunod patay</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>nouveau riche</t>
+          <t>dihard</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>['nakatugdon']</t>
+          <t>['lunod', 'patay']</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>"Ang mga tawo nga bag-o rang nakuhaan ug jackpot murag langaw nga nakatugdon sa kabaw."</t>
+          <t>Ang iyang amigo lunod patay sa iyang pagtuo bisan pa sa mga pagsulay.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Ang langaw naglupad-lupad sa palibot hangtod nakatugdon sa kabaw.</t>
+          <t>Ang sakayan ilang gisakyan nasangit sa dagkong balod, ug nahinumdom ko sa babaye nga lunod patay sa ubos sa dagat.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>madala nimo ang baka sa suba apan dili nimo mainom</t>
+          <t>manira sa dalan</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Mahimo nimong pagdala ang kabayo ngadto sa tubig</t>
+          <t>aron magpabilin nga magmata hangtod sa gabii</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>['madala', 'mainom']</t>
+          <t>['manira']</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Si Pedro giingnan nga bisan unsaon pagdasig, madala nimo ang baka sa suba apan dili nimo mainom.</t>
+          <t>Si Pedro pirmi manira sa dalan kada gabii.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Nagkakaboang ang mga mag-uuma kay madala nimo ang baka sa suba apan dili nimo mainom ang hayop bisan init kaayo ang adlaw.</t>
+          <t>Si Juan manira sa dalan aron mabantayan ang kalihokan sa mga dumuloong.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>halinon og aping</t>
+          <t>gwapo kon magtalikod</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>maayo kaayo nga hitsura</t>
+          <t>nindot nga tan-awon gikan sa likod</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>['halinon']</t>
+          <t>['magtalikod']</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Si Maria halinon og aping, daghan kaayo siya ug admirers.</t>
+          <t>Ang mga tao nga gwapo kon magtalikod kasagaran dili magdugay sa ilang relasyon.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Naghalinon og aping ang bata human siya gi-wash ug face ni Mama.</t>
+          <t>Si Juan gwapo kon magtalikod, kay nindot ug porma ang iyang buhok ug likod.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>gibuhi</t>
+          <t>mangnukos</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ang penis sa usa ka lalaki</t>
+          <t>sa pag-abli sa usa ka pista</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>['gibuhi']</t>
+          <t>['mangnukos']</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Gibuhi niya ang iyang mga tanom nga permi niyang ginatiman.</t>
+          <t>Si Juan giingnan nga dili mangnukos sa party sa iyang amiga.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>"Gibuhi sa amahan ang nawong sa iyang anak gamit ang panyo."</t>
+          <t>Ang iro misugod ug mangnukos sa iring nga mikarat sa atop.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>binuhi</t>
+          <t>murag langaw nga nakatugdon sa kabaw</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ang penis sa usa ka lalaki</t>
+          <t>nouveau riche</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['nakatugdon']</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Ang mga binuhi nga iro sa ilang balay kay puro mga pure breed.</t>
+          <t>"Ang mga bag-o rang nigraduate ug ni trabaho, murag langaw nga nakatugdon sa kabaw."</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Ang binuhi nga baka kay gi-atiman pag-ayo aron magamit sa umaabot nga negosyo sa gatas.</t>
+          <t>Natagbaw ang langaw ug tuas siya sa likod sa kabaw, murag langaw nga nakatugdon sa kabaw nga nagpangita ug pahulay.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>makakutaw og utok</t>
+          <t>gidaman</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>makapalibog</t>
+          <t>sa pag-aturog o pag-aturog</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>['makakutaw']</t>
+          <t>['gidaman']</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Ang explanation sa iyang professor makakutaw og utok kaayo.</t>
+          <t>"Kung mangutana ka og ing-ana, murag gidaman ka."</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Ang iyahang paghalo sa mainit nga supas makakutaw og utok kay wala pa man gud niupos ang kainit niini.</t>
+          <t>Pagmata nako sa buntag, nakita nako ang akong igsoon nga gidaman ug naglakaw-lakaw sa sala.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>manglutasay</t>
+          <t>ang baka nisulod sa kulon</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>usa ka manunulak sa mga bukog</t>
+          <t>gigamit sa pagsulti sa usa nga siya usa ka bakak o ikaw mahimo sa pagsulti sa laing nagbuwa</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>['manglutasay']</t>
+          <t>['nisulod']</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Si Juan giingnan nga manglutasay kay ang iyang uyab mas bata kaayo.</t>
+          <t>Sa dihang nagluto siya, naay baka nisulod sa kulon nga nagkalata.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Ang mga bata sa baryo magdula-dula ug manglutasay sa tabing-suba.</t>
+          <t>Naglibog ko pagtan-aw sa kusina kay ang baka gyud tinuod nga nisulod sa kulon.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>gi-indian</t>
+          <t>walay aso makumkom</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>sa tinuyo nga dili motuman sa usa ka appointment</t>
+          <t>walay sekreto nga magpabilin nga sekreto</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>['gi-indian']</t>
+          <t>['makumkom']</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Si Pedro gi-indian sa iyang uyab sa ilang sabot nga date.</t>
+          <t>Si Ana nakasabot nga walay aso makumkom, mao nga nagbantay siya sa iyang mga desisyon.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Wala moabot si Miguel sa ila nahuman nga sabot, kay gi-indian man siya sa Mindanao para magtuon sa mga lumad nga Indian didto.</t>
+          <t>Ang tinuod, bisan unsa ka kusog sa imong pagpaningkamot, walay aso makumkom basta maayo ang hangin.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>kuwang sa tagad</t>
+          <t>ul-ol</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>kinaiya sa usa ka nagpangita ug atensyon</t>
+          <t>sa pag- masturba Mga sinonim: batil</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>['tagad']</t>
+          <t>['ul-ol']</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Si Pedro kuwang sa tagad, bisan unsa nga event ganahan magpakita.</t>
+          <t>Ang iyang mga ul-ol nga istorya kay naghatag ug kalibog sa tanan.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Ang tanom nga wa matagda, nagpakita og mga sintomas nga kuwang sa tagad sama sa mga dili hapsay nga dahon.</t>
+          <t>Juan miingon nga siya gikapoy human siya mag-ul-ol sulod sa iyang kwarto.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>taliba</t>
+          <t>giprito sa kaugalingong mantika</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ang mga genital sa babaye</t>
+          <t>Alternatibo nga porma sa giluto sa kaugalingong mantika</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>['taliba']</t>
+          <t>['giprito']</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Ang mga pulis nag-taliba sa mga salida aron protektahan ang mga bisita.</t>
+          <t>Si Juan giprito sa kaugalingong mantika, kay nagpadayon sa iyang sayop.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Ang taliba nagsugod ug talagsaon nga lihok human sa pagkahuman sa operasyon.</t>
+          <t>Nagluto si Maria ug isda nga giprito sa kaugalingong mantika aron mas lami ang timpla.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>hatod og patay</t>
+          <t>maghilak ang adlaw</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>sa pagtambong sa usa ka paglubong o seremonya sa paghinumdom</t>
+          <t>mabul-og</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>['hatod', 'patay']</t>
+          <t>['maghilak']</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Si Pedro hatod og patay sa iyang kauban sa trabaho.</t>
+          <t>Ang mga tawo nag-relax sa balay samtang naghilak ang adlaw.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Nag-hatod og patay ang mga mag-uuma ngadto sa paglubong sa talis.</t>
+          <t>Ang mga bata nagdali og pauli pagkahuman nila makit-an nga maghilak ang adlaw tungod sa kusog nga ulan.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>makabugto og panty</t>
+          <t>higda sa lubi</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>pisikal o seksuwal nga madanihon</t>
+          <t>pag-ula</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>['makabugto']</t>
+          <t>['higda']</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Si Pedro ganahan kaayo sa iyang uyab kay makabugto og panty.</t>
+          <t>Si Juan higda sa lubi, pirmi lang maghubog-hubog.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Paglaba nako sa akong mga sinina, nasamad ang akong daliri tungod sa hugot nga elax na makabugto og panty.</t>
+          <t>Ang bata nakatulog ug higda sa lubi human magdula sa daplin sa baybayon.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>duwa og panit</t>
+          <t>pangatulig luwag</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>sa pag- masturba</t>
+          <t>gigamit sa pag-undang sa usa ka tawo nga misquoted o misheard sa usa ka gisulti</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>['duwa']</t>
+          <t>['pangatulig']</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Ang mga bata nga nagdula sa internet pirmi lang magduwa og panit.</t>
+          <t>"Pangatulig luwag imong mga ideas, kinahanglan pa nimo ug focus."</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Ang mga tambay sa kanto nagduwa og panit sa kadyot nga hagit sa ilang amigo.</t>
+          <t>"Sa kalit nga pangatulig luwag, nawad-an siya ug gana sa iyang gipangluto nga lugaw."</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>istorya ilalom sa dagat</t>
+          <t>ipanabi na sa clouds</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Usa ka dakong basura</t>
+          <t>Isulti kana sa mga marine</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['ipanabi']</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Ang mga tawo nga dili tinuod pirmi lang mag-istorya ilalom sa dagat.</t>
+          <t>Ang iyang mga istorya pirmi ipanabi na sa clouds kay dili tinuod.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Ang mga nanginhas nakadungog og istorya ilalom sa dagat samtang nagsubsob sa ilang buluhaton.</t>
+          <t>Ang mga piloto nagplano nga ipanabi na sa clouds ang mensahe nga nahuman na ang misyon.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>habwa ang kinaon</t>
+          <t>lisod pukawon ang gamata</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>pag-awhag</t>
+          <t>gigamit sa pagsulti sa nagmata o sa usa ka tawo nga dili magmata</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>['habwa', 'kinaon']</t>
+          <t>['pukawon']</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Si Maria naghabwa ang kinaon kay nagkalibanga.</t>
+          <t>Bisan unsaon, lisod pukawon ang gamata kung kapoy ang lawas.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Naghabwa ang bata sa kinaon gikan sa basket aron ipakaon sa mga iro.</t>
+          <t>Matag buntag, lisod pukawon ang gamata kay grabe ka duol ang ilang pagkatulog.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>litik</t>
+          <t>abot sa dalunggan ang ngisi</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>sa pag-aghat sa tudlo</t>
+          <t>nga dili gayod malipay</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>['litik']</t>
+          <t>['abot']</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Ang mga tawo nga naglitik sa ilang mga pangandoy kasagaran magmalampuson.</t>
+          <t>Ang bata, abot sa dalunggan ang ngisi sa dihang gihatagan ug dako nga regalo.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Naglingkod si Juan sa lamisa ug kalit niyang gilitik ang botelya nga nagbarog.</t>
+          <t>Ang babaye, abot sa dalunggan ang ngisi tungod sa iyang katawa.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>duwa og panit</t>
+          <t>bukhad og palad</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>sa pag- masturba</t>
+          <t>mahinatagon Synonyms: manggihatagon</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>['duwa']</t>
+          <t>['bukhad']</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Si Pedro walay laing gihimo kundi magduwa og panit pirmi.</t>
+          <t>Ang mga tao nga bukhad og palad kasagaran daghan ug mga amigo.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Gipakita sa maestro nga giunsa pagduwa og panit sa tambol aron makuha ang tukmang tingog.</t>
+          <t>Si Lola Juanita mihapit sa manghuhula aron pabasaon ang iyang bukhad nga palad.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>istorya ilalom sa dagat</t>
+          <t>dili makaon og iro</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Usa ka dakong basura</t>
+          <t>makalilisang</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['makaon']</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Ang iyang pangatarungan kay istorya ilalom sa dagat, walay klaro.</t>
+          <t>Ang iyang batasan dili makaon og iro, maong walay ganahan makighangyo niya.</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Ang mga diver nakahibalo nga lisud ang pag-istorya ilalom sa dagat tungod sa tubig.</t>
+          <t>Ang mga pagkaon nga gibutang sa lamesa dili makaon og iro kay peligroso kini sa ilang panglawas.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>kung wala kay lingaw sa kinabuhi, dakpa akong utot</t>
+          <t>ayaw adto og gubat kon wala kay bala</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>gigamit sa pag-undang sa usa ka nagpangita ug pagtagad</t>
+          <t>ayaw pagbuhat ug dili-andam</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>['lingaw', 'dakpa']</t>
+          <t>['adto']</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Kung wala kay lingaw sa kinabuhi, dakpa akong utot, kay walay lain maka-entertain nimo.</t>
+          <t>Ang mga negosyante giingnan nga ayaw adto og gubat kon wala kay bala sa kompetisyon.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Naglain akong tiyan, mao nga kung wala kay lingaw sa kinabuhi, dakpa akong utot aron makita nato ug tinuod ba.</t>
+          <t>Ang mga sundalo giingnan sa ilang kumander, "Ayaw adto og gubat kon wala kay bala, kay delikado ang kahimtang diha."</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>awas og palad</t>
+          <t>taga</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>• awasan og palad</t>
+          <t>pag-slash</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>['awas']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Si Ana awas og palad, maong pirmi lang maglisod bisan taas ang sweldo.</t>
+          <t>Ang mga kawatan nahadlok kay basin mataga sila sa mga tag-iya sa balay.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Gihugasan niya ang iyang palad ug karon nag-awas na ang tubig gikan niini.</t>
+          <t>Ang mananagat mihawid ug isda ug gitaga kini gamit ang sundang.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>hangyo kabayo</t>
+          <t>dili tanang butang sili nga mohalang dayon</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>usa ka maalamon nga paagi sa pagbaton ug usa ka butang</t>
+          <t>Dili tanan mahitabo sa usa ka higayon</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>['hangyo']</t>
+          <t>['mohalang']</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Ang mga tawo nga hangyo kabayo kasagaran magmalampuson sa ilang mga plano.</t>
+          <t>Ang mga tawo nga dili tanang butang sili nga mohalang dayon kasagaran magmalampuson sa ilang mga plano.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Ang bata naghangyo sa iyang ginikanan nga paliton siya og kabayo.</t>
+          <t>Nagpalit siya og daghang klase sa sili sa merkado, pero nakadiskubre siya nga dili tanang butang sili nga mohalang dayon.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>kung wala kay lingaw, dakpa akong utot</t>
+          <t>molayag sa kalipay</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>gigamit sa pag-undang sa usa ka nagpangita ug pagtagad</t>
+          <t>sa pagpakigsekso</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>['lingaw', 'dakpa']</t>
+          <t>['molayag']</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Kung wala kay lingaw, dakpa akong utot aron ma-testing nimo imong abilidad.</t>
+          <t>Ang mga amigo nagmolayag sa kalipay sa ilang road trip.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Paglingkod nako sa sofa, gisulti nako sa akong ig-agaw, "Kung wala kay lingaw, dakpa akong utot," aron makita namo kung makaya ba niya pagkakupot.</t>
+          <t>Ang mga bata nagmolayag sa kalipay samtang nagdula sa dagat sa buntag.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ander da bunal</t>
+          <t>ul-ol</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>gi-squeeze</t>
+          <t>sa pag- masturba Mga sinonim: batil</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>['bunal']</t>
+          <t>['ul-ol']</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Ang relasyon nila kay ander da bunal, maong klaro kaayo kinsa ang nagbuot.</t>
+          <t>Dili maayo nga magsige ka ug ul-ol kay makadaot kini sa imong reputation.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Ang bata misunod sa iyang mama nga "ander da bunal" human masagpaan ug kahoy.</t>
+          <t>"Ang bata natapolan ug dili gusto magtuon, murag ul-ol gyud siya."</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>tinagoan</t>
+          <t>gigukod sa plansa</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>gitago</t>
+          <t>ang usa ka tawo nga nagsul-ob ug mga sinina</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['gigukod']</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Ang tinagoan nga lihim ni Juan kay nahibaw-an na sa tanan.</t>
+          <t>Ang mga tawo nga gigukod sa plansa kasagaran dili mag-atiman sa ilang kaugalingon.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>"Ang tinagoan nga kwarta sa luyo sa aparador nadiskobrehan sa iyang igsoon."</t>
+          <t>Ganiha buntag, nagdali ko ug gamay, maong ang akong kamiseta gigukod sa plansa aron mawala ang tupi.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>mamalit og kaso</t>
+          <t>gwapa kon magtalikod</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>aron mahimong usa ka ambulance chaser</t>
+          <t>nindot nga tan-awon gikan sa likod</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['magtalikod']</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Ang mga tawo nga mamalit og kaso kasagaran mga abogado nga gustong magpasikat.</t>
+          <t>Ang mga tao nga gwapa kon magtalikod kasagaran maulaw kung mag-atubang.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Ang akong ig-agaw gusto mamalit og kaso aron magamit niya sa among eskwelahan nga praktis.</t>
+          <t>"Si Ana gwapa kon magtalikod kay nindot ug straight ang iyang buhok."</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>mabaw og kibot</t>
+          <t>tuslok baki</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>dali nga madaot</t>
+          <t>usa ka dula</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>['kibot']</t>
+          <t>['tuslok']</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Ang iyang kauban mabaw og kibot, bisan gamay lang nga butang maglagot na.</t>
+          <t>Ang tuslok baki kay usa ka traditional nga dula nga gipasa-pasa sa mga henerasyon.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Daling mobakwi si Ana kay mabaw og kibot, labi na kon naay kalit nga tingog.</t>
+          <t>Nagkagubot ang mga bata samtang nagtan-aw kung kinsa ang makatama sa baki sa ilang gipagawas nga tuslok.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>halinon og aping</t>
+          <t>kusog mokaon og gasolina</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>maayo kaayo nga hitsura</t>
+          <t>gas-gussing</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>['halinon']</t>
+          <t>['mokaon']</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Si Ana halinon og aping, daghan kaayo siya ug mga manliligaw.</t>
+          <t>Ang iyang motor kusog mokaon og gasolina, pirmi lang magpailis.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Nagposing si Ana aron makuhanan og halinon og aping nga larawan sa iyang mga album.</t>
+          <t>Nag-obserbar si Juan nga kusog mokaon og gasolina ang ilang makinarya sa umahan tungod kay daghan kaayong trabaho sa ting-ani.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>bukad og ngabil</t>
+          <t>magtumba og baka</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>mga labi nga may lapis</t>
+          <t>sa pag-ihaw sa usa ka vaca</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>['bukad']</t>
+          <t>['magtumba']</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Si Juan bukad og ngabil, bisan unsa nga istorya, pirmi lang magsige ug sulti.</t>
+          <t>Si Maria nalipay kay magtumba og baka ang iyang pamilya para sa pasko.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Ang bata kay bukad og ngabil tungod sa iyang allergies.</t>
+          <t>Ang mga trabahador sa uma magtumba og baka karong buntaga para sa karneng iprutos.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>mag-ihaw og lata</t>
+          <t>hangyo lubo</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>sa pagluto sa mga pagkaon nga tinago</t>
+          <t>usa ka hangyo nga gihimo sa ingon nga paagi nga dili kini makalikay</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>['mag-ihaw']</t>
+          <t>['hangyo', 'lubo']</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Ang mga estudyante kasagaran mag-ihaw og lata kung nagtipid.</t>
+          <t>Si Maria hangyo lubo, maong walay makatanggi sa iyang mga pangutana.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Si Lito nag-andam og dapog aron mag-ihaw og lata para sa ilang campfire na aktibidad.</t>
+          <t>Ang hangyo lubo ni Juan kay ang pagbahin sa iyang mga kalubian sa iyang mga silingan human sa bagyong miagi.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>kang kinsa man na imong sala</t>
+          <t>kapugngan pa ang baha, dili ang biga</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>gigamit sa pagsulti sa usa ka tawo nga sila lamang ang may sala sa ilang kaugalingon alang sa ilang kaugalingong mga problema</t>
+          <t>dili mapugngan</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>['sala']</t>
+          <t>['kapugngan']</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Kang kinsa man na imong sala nga gipaninguha nimo?</t>
+          <t>Si Maria adunay dakong pangandoy nga dili mapugngan, kapugngan pa ang baha, dili ang biga.</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>"Nagpangutana si Maria, 'Kang kinsa man na imong sala nga nasudlan?' kay wala siya nakasabot sa istorya."</t>
+          <t>Pag-abot sa kusog nga ulan, kapugngan pa ang baha, dili ang biga sa yuta nga grabe kaayo ang pag-inilog ug pag-atake.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>dugay pay manguros</t>
+          <t>buotan ra og matulog</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>usa ka piraso sa cake</t>
+          <t>malinong</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>['manguros']</t>
+          <t>['matulog']</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Si Juan dugay pay manguros kung magtrabaho sa opisina.</t>
+          <t>Ang mga bata nga buotan ra og matulog kasagaran magdala ug kasamok sa balay.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Buntag pa sa simbahan, dugay pay manguros ang mga tawo nga nagtipon sa una nga misa.</t>
+          <t>Si Lito, bisag buotan ra og matulog, abtik kaayo sa pagtrabaho kung alerto na.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>makakutaw og utok</t>
+          <t>magpalapad og papel</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>makapalibog</t>
+          <t>aron magbaton ug dungog sa buhat sa uban</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>['makakutaw']</t>
+          <t>['magpalapad']</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Si Maria nagreklamo kay ang instructions makakutaw og utok.</t>
+          <t>Ang iyang kauban sa trabaho pirmi magpalapad og papel sa mga achievements sa uban.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Si Maria nagdagan palibot sa lamisa nga makakutaw og utok.</t>
+          <t>Nagpalit siya og balayronon sa papel sa tindahan kay magpalapad siya og papel alang sa iyang project sa eskuwela.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>giluto sa kaugalingong mantika</t>
+          <t>sabong</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>sa pag-ukit sa kaugalingong lubnganan</t>
+          <t>usa ka kompetisyon</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>['giluto']</t>
+          <t>['sabong']</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Ang mga tawo nga magbuhat ug dautan kasagaran giluto sa kaugalingong mantika.</t>
+          <t>Ang mga manok nga ipangsabong kay gipangandaman ug maayo.</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Gihikay nila ang baboy sa pista ug giluto sa kaugalingong mantika.</t>
+          <t>Ang akong amahan mopalit og sabon sa merkado kay nahutdan na mi sa among balay.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>awas og palad</t>
+          <t>maabot sa luwa</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>• awasan og palad</t>
+          <t>duol dili layo</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>['awas']</t>
+          <t>['maabot']</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Ang mga awas og palad kasagaran maglisod sa kinabuhi kay dili kabalo magtipid.</t>
+          <t>Ang lugar nga ilang giadtoan kay maabot ra sa luwa, dili layo.</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Miuyog ko sa akong ulo nga dali ra kaayo nga awas ang palad sa baso.</t>
+          <t>Ang tubig nga akong gitilaw kay lami, hangtod maabot ra gyud sa luwa.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>magtumba og baka</t>
+          <t>agi sa bangag sa dagom</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>sa pag-ihaw sa usa ka vaca</t>
+          <t>pag-antos sa mga kalisdanan sa pagkab-ot sa imong tumong o damgo</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>['magtumba']</t>
+          <t>['agi']</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Si Maria nalipay kay magtumba og baka ang iyang pamilya para sa pasko.</t>
+          <t>Ang iyang negosyo agi sa bangag sa dagom bago niyag napalambo.</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Ang mga trabahador sa uma magtumba og baka karong buntaga para sa karneng iprutos.</t>
+          <t>Nagtan-aw siya unsaon pag-agi sa sinulid sa bangag sa dagom aron masugdan ang pagpanahi.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ang masuya madeads</t>
+          <t>ang baka nisulod sa kulon</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>gigamit sa pagsulti sa usa nga dili magkritika o magdumot sa gibuhat sa usa</t>
+          <t>gigamit sa pagsulti sa usa nga siya usa ka bakak o ikaw mahimo sa pagsulti sa laing nagbuwa</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>['masuya']</t>
+          <t>['nisulod']</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Ayaw suya-suya kay ang masuya madeads.</t>
+          <t>Sa dihang nag-away sila, mura'g baka nga nisulod sa kulon ang kasaba.</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Ang masuya madeads tungod kay nasuya siya sa bag-ong kotse sa iyang silingan ug naghinanok, naapsan siya sa sakuna.</t>
+          <t>Gikugang si Mama pagtan-aw niya nga ang baka tinuod gyud nga nisulod sa kulon.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>hunaw</t>
+          <t>ang masuya madeads</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>sa paghunaw sa kamot sa usa o sa uban</t>
+          <t>gigamit sa pagsulti sa usa nga dili magkritika o magdumot sa gibuhat sa usa</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>['hunaw']</t>
+          <t>['masuya']</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Si Juan naghunaw sa iyang responsibilidad sa trabaho.</t>
+          <t>Si Juan kay permi masuya sa mga gadgets sa uban, pero ang masuya madeads.</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Si Maria naghunaw sa iyang mga kamot human sa pagkaon.</t>
+          <t>Siya miingon nga ang masuya madeads, og nagtuo gyud siya nga ang pagkamasuya makaresulta sa pagkamatay.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>bunal</t>
+          <t>abot sa dunggan ang ngisi</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ang tungkod nga gigamit sa pag-atake o pag-bully sa usa ka hayop o tawo</t>
+          <t>nga dili gayod malipay</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>['bunal']</t>
+          <t>['abot']</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Ang mga bunal sa mga dula sa elementarya kay kasagaran gihimo ug kahoy.</t>
+          <t>Abot sa dunggan ang ngisi ni Manang Ines pagkakita sa iyang mga apo.</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Ang bunal nga gigamit sa mag-uuma kay gahi ug kahoy aron dili dali maguba.</t>
+          <t>Gani, abot sa dunggan ang ngisi ni Juan kay naputlan siya ug tabil sa iyang ngipon.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>kalas og bugo</t>
+          <t>makabugto og bra</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>usa ka pulong nga gigamit sa pagsulti sa usa ka tawo nga siya nagkinahanglan og dugay kaayo aron masabtan kon unsay gipamulong</t>
+          <t>pisikal o seksuwal nga madanihon</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>['kalas']</t>
+          <t>['makabugto']</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Ayaw pag-kalas og bugo, kay sayang lang ang imong panahon.</t>
+          <t>Si Juan ganahan kaayo sa iyang uyab kay makabugto og bra.</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Naglimpyo ko sa sala, unya kalas og bugo ang akong giusik kay naguba dayon ang dustpan.</t>
+          <t>"Ayoa pag-atiman sa imong sinina kay basin makabugto og bra ang lig-ag sa washing machine."</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>makabugto og panty</t>
+          <t>kulang sa dukol</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>pisikal o seksuwal nga madanihon</t>
+          <t>usa ka buangbuang nga tawo</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>['makabugto']</t>
+          <t>['dukol']</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Ang artista nga iyang nakita sa sine makabugto og panty gyud.</t>
+          <t>Si Juan kulang sa dukol, pirmi lang magtambay sa kanto.</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Ang hilo sa iyang bag-ong panty nipis ra kaayo nga dili kalikayan nga makabugto og panty kung mabira.</t>
+          <t>Si bata kulang sa dukol kay walay nag-amuma sa iya kabuang.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>bahong biyudo</t>
+          <t>gi-indian</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>adunay kusog nga baho nga musky o balsam</t>
+          <t>sa tinuyo nga dili motuman sa usa ka appointment</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>['bahong']</t>
+          <t>['gi-indian']</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Ang mga gamit sa balay nga wala gipanumbaling kay bahong biyudo.</t>
+          <t>Ang mga estudyante na gi-indian sa ilang maestra sa klase karon.</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Si Tatay Juan, nga usa ka biyudo, dili na makasabot sa bahong biyudo nga naggikan sa iyang mga sinina.</t>
+          <t>Siya gi-indian ang hilaw nga manok gamit ang tradisyonal nga resipe sa tribu.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>abot sa dunggan ang ngisi</t>
+          <t>habwa ang kinaon</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>nga dili gayod malipay</t>
+          <t>pag-awhag</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>['abot', 'dunggan', 'ngisi']</t>
+          <t>['habwa', 'kinaon']</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Sa dihang gihatagan siya ug award, abot sa dunggan ang ngisi ni Carla.</t>
+          <t>Ang iyang amiga naghabwa ang kinaon kay nasubraan ug kaon.</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Nagkatawa kaayo ang bata nga abot sa dunggan ang ngisi niya.</t>
+          <t>Ang bata naghabwa sa sudlanan aron makuha ang kinaon.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>pagtan-aw, kitkit langaw; paglingi, kitkit bungi</t>
+          <t>kulang sa dukol</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>gigamit nga isulti sa usa ka tawo nga imong gilimbongan sila sa pagtan-aw sa usa ka piho nga direksyon</t>
+          <t>usa ka buangbuang nga tawo</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>['kitkit', 'kitkit', 'bungi']</t>
+          <t>['dukol']</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>paglingi, kitkit bungi.</t>
+          <t>Ang iyang anak kulang sa dukol, dili gyud magtinarong sa pag-eskwela.</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Sa paghigda sa ilang balay, si Lito nakadungog ug sulti ni Jayjay nga "pagtan-aw, kitkit langaw; paglingi, kitkit bungi," ug nakatawa sila kay nasakpan tuod nga adunay langaw ug asong bungi sa may bintana.</t>
+          <t>Ang bata kulang sa dukol, mao nga giingnan siya sa iyang ginikanan nga magmatngon sa sunod nga dulaan.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>kulang sa tagad</t>
+          <t>ayaw pagbuot kay lain-lain ta og lubot</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>kinaiya sa usa ka nagpangita ug atensyon</t>
+          <t>ayaw ako isulti kon unsay buhaton</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>['tagad']</t>
+          <t>['pagbuot']</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Ang mga tawo nga kulang sa tagad kasagaran magbuhat ug dautan para makuha ang attention sa uban.</t>
+          <t>Ayaw pagbuot kay lain-lain ta og lubot, respetaray lang ta sa atong mga opinion.</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Ang bata kulang sa tagad kay wala siya gitagad sa mga tigulang samtang nagdula siya sa plasa.</t>
+          <t>Pagmeeting sa klase, nananghid si Junjun nga dili siya makagymnastics kay ingon niya, "Ayaw pagbuot kay lain-lain ta og lubot," nagsakit iyang lubot paglingkod.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ander da bunal</t>
+          <t>kuwang sa tagad</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>gi-squeeze</t>
+          <t>kinaiya sa usa ka nagpangita ug atensyon</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>['bunal']</t>
+          <t>['tagad']</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Ang ander da bunal nga bana kay kasagaran magpaubos ug musunod sa asawa.</t>
+          <t>Si Juan pirmi lang magpakita sa mga tao kay kuwang sa tagad.</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Si Lucas kay nagu-ander da bunal nga duwa, diin ang mga bata nagbungkag ug mga bulingon nga kahoy gamit ang bunal.</t>
+          <t>Ang bata nga nahibilin sa balay gamay ra kaayo ang nadawat nga kalooy, kuwang sa tagad sa iyang mga ginikanan.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>hangyo lubo</t>
+          <t>gisulod sa bulsa</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>usa ka hangyo nga gihimo sa ingon nga paagi nga dili kini makalikay</t>
+          <t>sa paglimbong</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>['hangyo', 'lubo']</t>
+          <t>['gisulod']</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Si Maria hangyo lubo, maong walay makatanggi sa iyang mga pangutana.</t>
+          <t>Si Maria gisulod sa bulsa, maong nag-antos siya sa iyang mga desisyon.</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Ang hangyo lubo ni Juan kay ang pagbahin sa iyang mga kalubian sa iyang mga silingan human sa bagyong miagi.</t>
+          <t>Gisulod ni Juan ang sensilyo sa iyang bulsa aron dili kini mawala.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>walay mahay nga gauna</t>
+          <t>gadalag uwan</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Ang nahimo dili mahimong malikayan</t>
+          <t>usa ka lalaki nga homoseksual</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>['mahay']</t>
+          <t>['nagdala']</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Ang mga estudyante giingnan nga walay mahay nga gauna, mao nga magtuon sila pag-ayo.</t>
+          <t>Ang iyang silingan gadalag uwan, pero respetado gihapon sa ilang lugar.</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Walay mahay nga gauna, mao nga si Ana karon nagbangutan tungod kay nawala ang iyang wallet.</t>
+          <t>Naglakaw kami sa kalsada ug nakita namo nga ang bata gadalag uwan aron dili mabasa sa kalit nga pag-abot sa ulan.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>gigukod sa plansa</t>
+          <t>maabot sa luwa</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ang usa ka tawo nga nagsul-ob ug mga sinina</t>
+          <t>duol dili layo</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>['gigukod']</t>
+          <t>['maabot']</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Ang mga tawo nga gigukod sa plansa kasagaran dili mag-atiman sa ilang kaugalingon.</t>
+          <t>Si Pedro pirmi lang maglakaw kay ang eskwelahan maabot ra sa luwa.</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Ganiha buntag, nagdali ko ug gamay, maong ang akong kamiseta gigukod sa plansa aron mawala ang tupi.</t>
+          <t>Ang lamesa natapsingan sa luwa ni Karen samtang siya nagtabi-tabi.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>murag gitilapan og iring</t>
+          <t>walay aso makumkom</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>walay sapayan</t>
+          <t>walay sekreto nga magpabilin nga sekreto</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>['gitilapan']</t>
+          <t>['makumkom']</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>"Ang iyang mga gamit sa opisina murag gitilapan og iring, limpyo ug hapsay."</t>
+          <t>Si Pedro nasayod nga walay aso makumkom, mao nga nagmatngon siya sa iyang mga lihok.</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>"Pagkakita nako sa lamisa, murag gitilapan og iring kay walay tanang bahaw nga niwangig."</t>
+          <t>Nagpayong si Anna duol sa siga apan nag-ingon siya nga walay aso makumkom tungod kay ihipan kini sa hangin.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>makabugto og bra</t>
+          <t>hangyo kabayo</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>pisikal o seksuwal nga madanihon</t>
+          <t>usa ka maalamon nga paagi sa pagbaton ug usa ka butang</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>['makabugto']</t>
+          <t>['hangyo']</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Si Juan ganahan kaayo sa iyang uyab kay makabugto og bra.</t>
+          <t>Ang iyang amiga hangyo kabayo, bisan unsa nga butang iyang makuha.</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>"Ayoa pag-atiman sa imong sinina kay basin makabugto og bra ang lig-ag sa washing machine."</t>
+          <t>Paghangyo siya sa presyo sa kabayo nga iyang gustong paliton.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>gigukod sa plansa</t>
+          <t>awas og palad</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ang usa ka tawo nga nagsul-ob ug mga sinina</t>
+          <t>• awasan og palad</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>['gigukod']</t>
+          <t>['awas']</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi lang gigukod sa plansa, bisan unsa nga sinina dili mahimutang.</t>
+          <t>Ang mga awas og palad kasagaran maglisod sa kinabuhi kay dili kabalo magtipid.</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Ang shirt ni Juan gigukod sa plansa human gilabhan.</t>
+          <t>Miuyog ko sa akong ulo nga dali ra kaayo nga awas ang palad sa baso.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>kung wala kay lingaw sa kinabuhi, dakpa akong utot</t>
+          <t>dili na nimo mabalik ang baha sa bukid</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>gigamit sa pag-undang sa usa ka nagpangita ug pagtagad</t>
+          <t>Ang nahimo nahimo na</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>['lingaw', 'dakpa']</t>
+          <t>['mabalik']</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Kung wala kay lingaw sa kinabuhi, dakpa akong utot, basi malingaw ka.</t>
+          <t>Si Ana nakasabot nga dili na nimo mabalik ang baha sa bukid, mao nga nag-move on na siya.</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Nagduwa ang mga bata og palumba sa iskina ug miingon si Juan, "Kung wala kay lingaw sa kinabuhi, dakpa akong utot, paglingaw-lingaw lang."</t>
+          <t>Nagbaha sa bukid tungod sa kusog nga ulan, ug bisan unsaon pa nimo og paningkamot, dili na nimo mabalik ang baha sa bukid nga ubos.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>pasok, Luningning</t>
+          <t>ang gaba dili magsaba</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>miingon sa kaugalingon sa dihang pag-poking sa usa sa iyang mga winnings sa usa ka dula sa mga kard</t>
+          <t>ang silot tungod sa iyang mga sayop o mga paglapas moabut sa wala damha</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>['pasok']</t>
+          <t>['magsaba']</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Pasok, Luningning, kay daghan pa ta ug buhaton.</t>
+          <t>Si Pedro nabulabog kay nasuko ang iyang giilad, ang gaba dili magsaba.</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Nangabli si Luningning sa pultahan ug giingnan siya sa iyang mama, "Pasok, Luningning, kay ulan kaayo sa gawas."</t>
+          <t>Sa kalit nga pagtandog sa kanal, nabali ang sungkod ni Lito ug nahangit siya, gipakita nga ang gaba dili magsaba.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>dili na mabalik ang baha paingon sa bukid</t>
+          <t>kuyog baboy</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Ang nahimo dili mahimong malikayan</t>
+          <t>usa ka tagalong</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>['mabalik']</t>
+          <t>['kuyog']</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Si Juan nasayod nga dili na mabalik ang baha paingon sa bukid, mao nga nagpadayon na siya.</t>
+          <t>Si Maria pirmi lang kuyog baboy, bisan asa moadto iyang best friend naa gyud.</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Ang mga lumulupyo sa baryo nahibulong kay dili na mabalik ang baha paingon sa bukid bisan sa kusog nga ulan.</t>
+          <t>Naglaag mi sa uma ug nagdala mi og kuyog baboy aron makalingaw ang mga bata.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>nakalugsong</t>
+          <t>gwapo kon magtalikod</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>sa pag-adto gikan</t>
+          <t>nindot nga tan-awon gikan sa likod</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>['nakalugsong']</t>
+          <t>['magtalikod']</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Nakalugsong na mi ug gidalit ang among mga ani sa lungsod.</t>
+          <t>Ang iyang amigo gwapo kon magtalikod, pero bati diay pagtan-aw sa iyang nawong.</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Naglakaw mi sa bukid ug nakalugsong mi ngadto sa suba para maligo.</t>
+          <t>Nagpicture ko sa akong iro sa dagat, ug gwapo kon magtalikod kay nindot kaayo iyang itom nga balhibo sa likod.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>lamoy</t>
+          <t>gi-indian</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>pag-abot</t>
+          <t>sa tinuyo nga dili motuman sa usa ka appointment</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>['lamoy']</t>
+          <t>['gi-indian']</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>"Lamoya nalang na imong gibuhat, walay gamit."</t>
+          <t>Si Juan gi-indian sa iyang kliyente sa ilang appointment.</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>"Gi-lamoy sa bata ang dakong pan nakon."</t>
+          <t>Siya gidala sa pagtuon ang mga katigulangan nga gi-indian ni Magellan sa Sugbo kaniadto.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>bahong biyudo</t>
+          <t>ayaw pagbuot, lain-lain tag lubot</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>adunay kusog nga baho nga musky o balsam</t>
+          <t>ayaw ako isulti kon unsay buhaton</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>['bahong']</t>
+          <t>['pagbuot']</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Ang iyang sinina nga bahong biyudo kay dili nimo malapasan.</t>
+          <t>Lain-lain tag lubot, mao nga kinahanglan respetuhon ang desisyon sa uban.</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Nahibulong mi ngano'ng bahong biyudo siya apan wala diay siya'y asawa nga namatay.</t>
+          <t>Sa klase sa Biology, gitun-an namo nga lain-lain og porma ang lubot sa matag matang sa hayop.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>giprito sa kaugalingong mantika</t>
+          <t>kuwang sa tagad</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Alternatibo nga porma sa giluto sa kaugalingong mantika</t>
+          <t>kinaiya sa usa ka nagpangita ug atensyon</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>['giprito']</t>
+          <t>['tagad']</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Si Juan giprito sa kaugalingong mantika, kay nagpadayon sa iyang sayop.</t>
+          <t>Si Pedro kuwang sa tagad, bisan unsa nga event ganahan magpakita.</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Nagluto si Maria ug isda nga giprito sa kaugalingong mantika aron mas lami ang timpla.</t>
+          <t>Ang tanom nga wa matagda, nagpakita og mga sintomas nga kuwang sa tagad sama sa mga dili hapsay nga dahon.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>agi sa bangag sa dagom</t>
+          <t>gigukod sa sudlay</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>pag-antos sa mga kalisdanan sa pagkab-ot sa imong tumong o damgo</t>
+          <t>nga walay buhok</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>['agi', 'bangag']</t>
+          <t>['gigukod']</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Ang ilang proyekto agi sa bangag sa dagom sa kalisod.</t>
+          <t>Si Pedro pirmi lang gigukod sa sudlay, bisan unsa nga event, dili mag-comb.</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Ipasulod ni Maria ang sinulid agi sa bangag sa dagom aron makatahi siya og sinina.</t>
+          <t>Anaa sa lamesa ang sudlay nga gigukod sa mga bata samtang nagdula sila.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>murag namatyag iring</t>
+          <t>makakutaw og utok</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>gigamit sa paghulagway sa usa ka tawo nga nagtangis nga nagtangis o nagtangis nga nagtangis</t>
+          <t>makapalibog</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>['namatyag']</t>
+          <t>['makakutaw']</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>"Ang bata murag namatyag iring, hilak kaayo pagnalaya."</t>
+          <t>Ang explanation sa iyang professor makakutaw og utok kaayo.</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Ang iring sa atop murag namatyag iring, kusog kaayo ang pangubog.</t>
+          <t>Ang iyahang paghalo sa mainit nga supas makakutaw og utok kay wala pa man gud niupos ang kainit niini.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>sabong</t>
+          <t>pangatulig luwag</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>usa ka kompetisyon</t>
+          <t>gigamit sa pag-undang sa usa ka tawo nga misquoted o misheard sa usa ka gisulti</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>['sabong']</t>
+          <t>['pangatulig']</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Ang mga manok nga ipangsabong kay gipangandaman ug maayo.</t>
+          <t>"Pangatulig luwag imong mga plano, walay klaro."</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Ang akong amahan mopalit og sabon sa merkado kay nahutdan na mi sa among balay.</t>
+          <t>Ang iyang pangatulig luwag kay naguba tungod sa karaan na kaayo nga kaldero.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>manira sa dalan</t>
+          <t>pangatulig luwag</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>aron magpabilin nga magmata hangtod sa gabii</t>
+          <t>gigamit sa pag-undang sa usa ka tawo nga misquoted o misheard sa usa ka gisulti</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['pangatulig']</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>"Ayaw pag manira sa dalan, naa pa kay buhaton."</t>
+          <t>Ang iyang plano kay murag pangatulig luwag, walay klaro nga direksyon.</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Ang mga tindahan manira sa dalan matag alas-otso sa gabi-i.</t>
+          <t>"Human sila pagkutaw sa sabaw, nag-pangatulig luwag dayon aron limpyo ang gamit."</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>kulang sa dukol</t>
+          <t>gwapo kon magtalikod</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>usa ka buangbuang nga tawo</t>
+          <t>nindot nga tan-awon gikan sa likod</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>['dukol']</t>
+          <t>['magtalikod']</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Si Maria kulang sa dukol, pirmi lang magbulakbol.</t>
+          <t>Si Juan gwapo kon magtalikod, pero dili na kaayo pag-atubang.</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Ang bata kulang sa dukol sa iyang likod kay nagtambay ra sa duyan.</t>
+          <t>Nagkatawa si Ana kay ang iyang iro gwapo kon magtalikod sa iyang fluffy nga ikog.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>miulbo ang kaspa</t>
+          <t>mogawas ang pari nga walay ulo</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>sa pag-abli ngadto sa kasuko</t>
+          <t>gigamit sa paghadlok sa mga bata gikan sa mga samad</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['mogawas']</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Si Ana miulbo ang kaspa human nabal-an nga gilimbongan siya.</t>
+          <t>Mogawas ang pari nga walay ulo kuno kung aduna'y mamatay sa baryo.</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Human sa dugang duha ka adlaw nga walay ligo, si Pedro nakabantay nga miulbo ang kaspa sa iyang ulo.</t>
+          <t>Sa halangdong sugilanon, kon malangan ang mga novena sa alas dose sa kagabhion, mosulod ang pari nga walay ulo sa simbahan ug mopahimangno sa mga tawo.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ipanabi na sa clouds</t>
+          <t>gibati og kaanyag</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Isulti kana sa mga marine</t>
+          <t>prima donna</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>['ipanabi']</t>
+          <t>['gibati']</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Ayaw na lang pagsabot ana, ipanabi na sa clouds.</t>
+          <t>Si Ana gibati og kaanyag, maong pirmi siya nagbuot-buot.</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Pagka-adlaw nga hayag, naglingkod si Maria sa atop ug gusto niyang pasundayag sa iyang gibati, busa iyang giingon sa iyang kaugalingon, "Ipanabi na sa clouds ang akong kalipay."</t>
+          <t>"Gibati gyud ni Carla og kaanyag sa iyang bag-ong sinina, maong nagpakita siya sa iyang mga higala."</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>lapos sa pikas dunggan</t>
+          <t>murag langaw nga nakatugdon sa kabaw</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>sa pagsulod sa usa ka dalunggan ug paggawas sa laing dalunggan</t>
+          <t>nouveau riche</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>['lapos', 'dunggan']</t>
+          <t>['nakatugdon']</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Ang tambag sa iyang ginikanan lapos ra sa pikas dunggan.</t>
+          <t>"Si Ana, gikan sa pagka-pobre, murag langaw nga nakatugdon sa kabaw karon."</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Nakita namo ang gamay nga sungo nga giigo sa bala, naglapos gyud sa pikas dunggan.</t>
+          <t>"Nagtan-aw ko sa uma ug nakita nako nga murag langaw nga nakatugdon sa kabaw."</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>habwa ang kinaon</t>
+          <t>kung wala kay lingaw sa kinabuhi, dakpa akong utot</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>pag-awhag</t>
+          <t>gigamit sa pag-undang sa usa ka nagpangita ug pagtagad</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>['habwa', 'kinaon']</t>
+          <t>['dakpa']</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Si Pedro naghabwa ang kinaon kay nasuka.</t>
+          <t>Kung wala kay lingaw sa kinabuhi, dakpa akong utot, tan-awon nato unsay imong mahimo.</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Naglimpyo si Maria sa kusina ug iyang gihabwa ang kinaon sa lamisa human sa ilang paniudto.</t>
+          <t>Naglingkod siya sa sala, dayon gisulti niya, "Kung wala kay lingaw sa kinabuhi, dakpa akong utot," samtang nangipi siya paglingaw-lingaw.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>bibingkang liki</t>
+          <t>dili na mabalik ang baha paingon sa bukid</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>ang mga genital sa babaye</t>
+          <t>Ang nahimo dili mahimong malikayan</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>['liki']</t>
+          <t>['mabalik']</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Si Pedro nagpakatawa sa mga barkada gamit ang bibingkang liki nga istorya.</t>
+          <t>Ang mga tawo giingnan nga dili na mabalik ang baha paingon sa bukid, mao nga nag-move on na.</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Nag-andam si Lola Maria og bibingkang liki alang sa Pasko.</t>
+          <t>Pag-abot sa panahon sa tig-ulan, diha ra jud sa patag magtapok ang tubig kay dili na mabalik ang baha paingon sa bukid.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ander de bunal</t>
+          <t>murag namiya og tai</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>gi-squeeze</t>
+          <t>Usa ka tawo nga mibiya sa dili-iasa nga walay iyang pulong</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>['bunal']</t>
+          <t>['namiya']</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Ang mga ander de bunal kay dili na maghunahuna sa ilang kaugalingong gusto.</t>
+          <t>"Si Ana murag namiya og tai, wala na gani nagpahibalo sa iyang mga plano."</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Si Andres kay nanghita og bunal ug gahapon gi-install niya ang iyang ander de bunal sa likod sa balay.</t>
+          <t>"Nakita nako si Tomas nga nagdali-dali padung sa banyo, murag namiya og tai."</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>baba sa atay</t>
+          <t>gilawog sa tirong</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ang diaphragm</t>
+          <t>sa pagbutang sa peligro sa usa ka tawo, ilabina</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>['baba']</t>
+          <t>['gilawog']</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Ang mga tambal para sa baba sa atay kay kinahanglan sa pag-maintain sa maayong kondisyon.</t>
+          <t>Si Pedro gilawog sa tirong sa iyang kauban, maong nasakpan sa ilang boss.</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>"Pagkalami gyud sa adobo nga akong giandam, labi na ang baba sa atay nga humok ug lami."</t>
+          <t>Gibantayan namo ang iring samtang gilawog namo kini sa tirong diha sa suba.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>molayag sa kalipay</t>
+          <t>mangayo og manghod</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>sa pagpakigsekso</t>
+          <t>usa ka kaso sa bata nga nag-asuso o nag-agom sa iyang mga tudlo</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>['molayag']</t>
+          <t>['mangayo']</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Ang mga magkauban nagmolayag sa kalipay sa ilang outing sa beach.</t>
+          <t>Si Pedro nakakita sa iyang anak nga mangayo og manghod sa iyang tiil.</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Ang mga langgam nagmolayag sa kalipay sa kataas-kataas nga kahoy.</t>
+          <t>"Mangayo og manghod si Maria kay gusto siya ug uska mubo nga bunal sa nakatigulang."</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>dili na mabalik ang baha paingon sa bukid</t>
+          <t>gwapa kon magtalikod</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Ang nahimo dili mahimong malikayan</t>
+          <t>nindot nga tan-awon gikan sa likod</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>['mabalik']</t>
+          <t>['magtalikod']</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Ang mga estudyante nakabalo nga dili na mabalik ang baha paingon sa bukid, mao nga nagplano na sila pag-ayo.</t>
+          <t>Ang iyang kauban sa trabaho gwapa kon magtalikod, pero pag-atubang, dili na diay.</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Pagkahuman sa kusog nga ulan, ang mga taga-barangay nag-istorya nga bisan unsaon pa, dili na mabalik ang baha paingon sa bukid, kay daghan kaayo ang tubig nga midiretso sa dagat.</t>
+          <t>Sa daghan nilang mga selfie, gwapa kon magtalikod si Ana, apan mas gwapa pag-atubang.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>lamoy</t>
+          <t>mangayo og manghod</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>pag-abot</t>
+          <t>usa ka kaso sa bata nga nag-asuso o nag-agom sa iyang mga tudlo</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>['lamoy']</t>
+          <t>['mangayo']</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>"Si Ana, sige lang lamoy walay klaro."</t>
+          <t>Si Juan nalipay kay ang iyang baby nakakat-on nga mangayo og manghod.</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>"Ang bata malipayon nga naglamoy sa iyang paborito nga tsokolate."</t>
+          <t>"Si Maria nangayo og manghod kay kini ang gipangita sa ilahang tapok."</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>kirig</t>
+          <t>agi sa bangag sa dagom</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>pag-awhag</t>
+          <t>pag-antos sa mga kalisdanan sa pagkab-ot sa imong tumong o damgo</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>['kirig']</t>
+          <t>['agi']</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Si Juan kirig sa kahadlok pagkakita sa aksidente.</t>
+          <t>Ang ilang relasyon agi sa bangag sa dagom sa daghang pagsulay.</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Si Maria kirig samtang gidalikyat siya sa ospital tungod sa iyang sakit.</t>
+          <t>Ang karayom wala pa maagi ug hilo kay gahi jud ang pag-agi sa bangag sa dagom.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>duwa og panit</t>
+          <t>makabugto og panty</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>sa pag- masturba</t>
+          <t>pisikal o seksuwal nga madanihon</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>['duwa']</t>
+          <t>['makabugto']</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Ang iyang mga kauban sa trabaho pirmi lang magbinuang ug magduwa og panit.</t>
+          <t>Si Pedro ganahan kaayo sa iyang uyab kay makabugto og panty.</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Ang mga bata nangita og bola aron makaduwa og panit sa basketball court.</t>
+          <t>Paglaba nako sa akong mga sinina, nasamad ang akong daliri tungod sa hugot nga elax na makabugto og panty.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ipanabi na sa clouds</t>
+          <t>paabang</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Isulti kana sa mga marine</t>
+          <t>pag-abang</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>['ipanabi']</t>
+          <t>['paabang']</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Kung gusto ka maabot ang imong damgo, ipanabi na sa clouds.</t>
+          <t>Ang ilang negosyo nga paabang og sakyanan kay booming na kaayo karon.</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>"Ang mensahe gikan sa iyang email kay ipanabi na sa clouds para dali ra mag-access bisan asa."</t>
+          <t>Nagpaabang sila og kwarto sa ilang balay alang sa mga turista.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>babayeng ikogan</t>
+          <t>hunaw</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>transgender</t>
+          <t>sa paghunaw sa kamot sa usa o sa uban</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>['ikogan']</t>
+          <t>['hunaw']</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Si Ana nga babayeng ikogan kay walay klaro nga direksyon sa kinabuhi.</t>
+          <t>Si Maria naghunaw sa iyang mga sala aron dili siya mahatagan ug parusa.</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Ang babayeng ikogan sa sirkus mao'y nagdala og daghang tawo kay talagsaon siya.</t>
+          <t>Gihunaw ni Juan ang iyang mga kamot human sa pagkaon.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>manira sa dalan</t>
+          <t>lisod pukawon ang gamata</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>aron magpabilin nga magmata hangtod sa gabii</t>
+          <t>gigamit sa pagsulti sa nagmata o sa usa ka tawo nga dili magmata</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['pukawon']</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Ang mga batan-on kasagaran manira sa dalan kung walay lingaw.</t>
+          <t>Lisod pukawon ang gamata, labi na kung bugnaw ang panahon.</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Ang tindero manira sa dalan kung udto kay init na kaayo.</t>
+          <t>"Nakita nako nga lisod pukawon ang gamata kay nagkatulog pa gyud siya ug maayo."</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>mura og halas nga nagluno</t>
+          <t>kirig</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>ang usa ka tawo nga magbiya sa iyang mahugaw nga sinina sa tanang dapit sa balay</t>
+          <t>pag-awhag</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>['nagluno']</t>
+          <t>['kirig']</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>"Ang silingan namo mura og halas nga nagluno, walay tarong pagbutang sa mga gamit."</t>
+          <t>Si Juan kirig sa kahadlok pagkakita sa aksidente.</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Ang among iring gibantayan kaayo ang halas nga nagluno sa halang nga sagbot sa among jardin.</t>
+          <t>Si Maria kirig samtang gidalikyat siya sa ospital tungod sa iyang sakit.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ipanabi na sa clouds</t>
+          <t>ang baka nisulod sa kulon</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Isulti kana sa mga marine</t>
+          <t>gigamit sa pagsulti sa usa nga siya usa ka bakak o ikaw mahimo sa pagsulti sa laing nagbuwa</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>['ipanabi']</t>
+          <t>['nisulod']</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Ipanabi na sa clouds ang imong mga tinguha ug siguroha nga mo-trabaho ka para ana.</t>
+          <t>Ang pagplano nila nga walay klaro mura'g baka nga nisulod sa kulon.</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Nakita nako ang bata nga naglingkod sa atop sanglit gilabay niya ang iyang mensahe ug ipanabi na sa clouds.</t>
+          <t>Ang bata nalipay kay nakita niya nga ang baka nisulod sa kulon sa pagdula-dula.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ipanabi na sa clouds</t>
+          <t>mag-ugbok og mohon</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Isulti kana sa mga marine</t>
+          <t>sa pagpakigsekso</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>['ipanabi']</t>
+          <t>['mag-ugbok']</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Bisan unsa ka lisod, ipanabi na sa clouds ang imong mga pag-ampo.</t>
+          <t>Si Maria ug ang iyang bana mag-ugbok og mohon sa ilang balay.</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Pagka gabii, among ipanabi na sa clouds ang among mga mensahe pinaagi sa drone nga adunay mga light display.</t>
+          <t>Ang mga trabahante mag-ugbok og mohon aron masugdan na ang pagtukod sa bag-ong balay.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>dula og panit</t>
+          <t>mag-ugbok og mohon</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>sa pag- masturba</t>
+          <t>sa pagpakigsekso</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>['dula']</t>
+          <t>['mag-ugbok']</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Si Juan dula og panit, pirmi lang magtambay ug magbuot-buot.</t>
+          <t>Si Pedro nagplano nga mag-ugbok og mohon human sa kasal.</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Si Ana migamit og kutsilyo aron dulaon ang panit sa mansanas.</t>
+          <t>Ang mga mag-uuma mag-ugbok og mohon aron markahan ang yuta nga ilang bungahon.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>anak sa sala</t>
+          <t>ayaw pagbuot kay lain-lain ta og lubot</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>usa ka anak nga dili-konsejero</t>
+          <t>ayaw ako isulti kon unsay buhaton</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>['sala']</t>
+          <t>['pagbuot']</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Ang anak sa sala kasagaran maglisod sa pagsulod sa mga respetadong institusyon.</t>
+          <t>Dili tanan magkauyon, kay lain-lain ta og lubot.</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Nagbisita ang pari sa balay ug giampo ang anak sa sala nga nakabaton og sakit.</t>
+          <t>Sa baki sa klase, si Ma'am Ana nagtudlo nga lain-lain ta og lubot depende sa atong klase sa pagkaon ug mga gawi.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>lapos sa pikas dunggan</t>
+          <t>agi sa bangag sa dagom</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>sa pagsulod sa usa ka dalunggan ug paggawas sa laing dalunggan</t>
+          <t>pag-antos sa mga kalisdanan sa pagkab-ot sa imong tumong o damgo</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>['lapos', 'dunggan']</t>
+          <t>['agi']</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Si Pedro pirmi lang lapos sa pikas dunggan ang mga lectures sa eskwela.</t>
+          <t>Si Pedro agi sa bangag sa dagom aron lang makapasar sa eksam.</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Si Juan nagkagubot ang buhok kay naay langaw nga misulod sa iyang dunggan ug nilapos sa pikas dunggan.</t>
+          <t>Si Maria naglisod og pagsulod sa pisi agi sa bangag sa dagom samtang nagpanahi siya og sinina.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>kakha tuka</t>
+          <t>abot sa dunggan ang ngisi</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>kamot-sa-lubong</t>
+          <t>nga dili gayod malipay</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>['kakha', 'tuka']</t>
+          <t>['abot']</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Si Juan pirmi lang kakha tuka, walay nahabilin nga budget.</t>
+          <t>Abot sa dunggan ang ngisi ni Lito pagkakita sa iyang paboritong artista.</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Ang maya nagkakha tuka sa nataran.</t>
+          <t>Nagpanglingo si Ana kay abot sa dunggan ang iyang ngisi sa paglingaw sa sayop nga katawa ni Juan.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>abot sa dalunggan ang ngisi</t>
+          <t>dili na mabalik ang baha paingon sa bukid</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>nga dili gayod malipay</t>
+          <t>Ang nahimo dili mahimong malikayan</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>['abot', 'dalunggan', 'ngisi']</t>
+          <t>['mabalik']</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Pagkahuman sa eksam, abot sa dalunggan ang ngisi ni Juan kay nakapasar siya.</t>
+          <t>Si Ana nakasabot nga dili na mabalik ang baha paingon sa bukid, mao nga nag-move on na sa iyang kinabuhi.</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Nagtan-aw ko sa litrato nga gipakita ni Ana, abot sa dalunggan ang ngisi niya sa kalipay.</t>
+          <t>Human sa kusog nga ulan, nasayod na ang mga residente nga dili na gyud mabalik ang baha paingon sa bukid, busa nanginahanglan gyud silang mag-andam sa umaabot nga panahon.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ul-ol</t>
+          <t>ipanabi na sa clouds</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>sa pag- masturba Mga sinonim: batil</t>
+          <t>Isulti kana sa mga marine</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>['ul-ol']</t>
+          <t>['ipanabi']</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Ang iyang mga ul-ol nga istorya kay naghatag ug kalibog sa tanan.</t>
+          <t>Ang imong mga plano, ipanabi na sa clouds kay maabot ra na.</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Juan miingon nga siya gikapoy human siya mag-ul-ol sulod sa iyang kwarto.</t>
+          <t>Ang detalye sa imong presentation, ipanabi na sa clouds aron ma-access sa tanan bisan asa pa.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>mangayo og manghod</t>
+          <t>ipanabi na sa clouds</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>usa ka kaso sa bata nga nag-asuso o nag-agom sa iyang mga tudlo</t>
+          <t>Isulti kana sa mga marine</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>['mangayo']</t>
+          <t>['ipanabi']</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Ang mga bata nga mangayo og manghod kasagaran mga healthy nga bata.</t>
+          <t>Ang imong mga pangandoy, ipanabi na sa clouds aron matinuod.</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Ang magtiayon midesisyon nga mangayo og manghod kay gusto nila dungagan ang ilang pamilya.</t>
+          <t>Gusto nakong ipaabot ang akong mensahe sa mga higala ko nga naa sa layo, mao nga ipanabi na sa clouds pinaagi sa teknolohiya.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>duwa og panit</t>
+          <t>gi-indian</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>sa pag- masturba</t>
+          <t>sa tinuyo nga dili motuman sa usa ka appointment</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>['duwa']</t>
+          <t>['gi-indian']</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Si Maria naglagot kay si Juan pirmi lang magduwa og panit bisan kinahanglanon siya.</t>
+          <t>Si Pedro gi-indian sa iyang uyab sa ilang sabot nga date.</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Nagpraktis ang mga bata nga magduwa og panit para sa ilang teatro sa eskuwela.</t>
+          <t>Wala moabot si Miguel sa ila nahuman nga sabot, kay gi-indian man siya sa Mindanao para magtuon sa mga lumad nga Indian didto.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>hilawas</t>
+          <t>kapugngan pa ang baha, dili ang biga</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>coitus</t>
+          <t>dili mapugngan</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['kapugngan']</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Ang hilawas nga kinabuhi kay wala'y klaro nga padulngan.</t>
+          <t>Ang iyang kalagot dili mapugngan, kapugngan pa ang baha, dili ang biga.</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>"Nagkinahanglan ang bata og hilawas nga panginahanglanon arun maatiman ang iyang kalawasan."</t>
+          <t>Sa kadako sa kusog sa ulan, kapugngan pa ang baha, dili ang biga nga gihunahuna sa mga tao.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>tuslok baki</t>
+          <t>buotan ra og matulog</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>usa ka dula</t>
+          <t>malinong</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>['tuslok']</t>
+          <t>['matulog']</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Ang mga bata nagpraktis sa tuslok baki aron mahimong champion sa dula.</t>
+          <t>Ang iyang anak buotan ra og matulog, kay pirmi lang mangaway sa mga silingan.</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>"Nakit-an nako si Lito nga nagkuha og sungkod aron magtuslok baki sa daplin sa sapa."</t>
+          <t>Gabiina na kaayo ug buotan ra og matulog ang bata sa ilang kwarto.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>manakop og ligid</t>
+          <t>taliba</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>nga ang usa ka tawo naugtang sa usa ka sakyanan</t>
+          <t>ang mga genital sa babaye</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>['manakop', 'ligid']</t>
+          <t>['taliba']</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Si Pedro manakop og ligid kay nagdagan-dagan sa kalsada.</t>
+          <t>Ang mga pulis nag-taliba sa mga salida aron protektahan ang mga bisita.</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Nagdula mi og dakop-dakop sa plaza unya nakalingkod ko para mopahuway, apan kalit nga miingon ang akong amigo nga manakop og ligid mi sa mga sakyanan nga nag-agi atubangan sa balay.</t>
+          <t>Ang taliba nagsugod ug talagsaon nga lihok human sa pagkahuman sa operasyon.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>kulang sa dukol</t>
+          <t>pasok, Luningning</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>usa ka buangbuang nga tawo</t>
+          <t>miingon sa kaugalingon sa dihang pag-poking sa usa sa iyang mga winnings sa usa ka dula sa mga kard</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>['dukol']</t>
+          <t>['pasok']</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Si Pedro kulang sa dukol, maong pirmi lang magbinuang.</t>
+          <t>Pasok, Luningning, ug paminawa ang mga instructions.</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Ang bata kulang sa dukol, mao nga ipatuli pa siya karong bulan para sakto ug kompleto.</t>
+          <t>"Pasok, Luningning, kay naghulat na ang imong amahan sa kusina."</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>hilawas</t>
+          <t>sabong</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>coitus</t>
+          <t>usa ka kompetisyon</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['sabong']</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Ang hilawas nga relasyon sa diha nga walay commitment kay lisod.</t>
+          <t>Ang sabong sa mga manok kay paborito nga pastime sa mga kalalakin-an.</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Nagkinahanglan ko ug hilawas nga pagkaon aron magpabiling lig-on ug himsog ang lawas.</t>
+          <t>Nagbutang kog tubig ug sabong sa palanggana para sa laba.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>bahong biyuda</t>
+          <t>bisan ang kabaw nga naay upat ka tiil masipyat</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>adunay kusog nga baho nga musky o balsam</t>
+          <t>kitang tanan magkamali</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>['bahong', 'biyuda']</t>
+          <t>['naay', 'masipyat']</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Si Juan bahong biyuda kay wala gyud maligo ug maayo.</t>
+          <t>Si Pedro nasipyat sa exam, bisan ang kabaw nga naay upat ka tiil masipyat.</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Ang akong silingan nga si Maria, nga dugay nang biyuda, miingon nga dili siya gusto og bahong biyuda sa iyang sinina.</t>
+          <t>Sa among bukid, nakita nako nga bisan ang kabaw nga naay upat ka tiil masipyat ug mulakaw diha sa dili patag nga dalan.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>pabuto</t>
+          <t>tuslok baki</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>usa ka patok</t>
+          <t>usa ka dula</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>['pabuto']</t>
+          <t>['tuslok']</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Ang mga bata malipay kaayo sa mga pabuto kada New Year.</t>
+          <t>Ang mga bata nagpraktis sa tuslok baki aron mahimong champion sa dula.</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Nagpalit kami og daghang pabuto para sa pista sa baryo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>hilawas</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>coitus</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>Ang mga tawo nga maghilawas kay kasagaran mahadlok magcommit.</t>
-        </is>
-      </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>Ang lami sa hilawas nga prutas kay wala'y sama.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>paabang</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>pag-abang</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>Gipahimutang ang iyang balay aron ipaabang sa mga bakasyonista.</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>Nagpaabang sila og mga bisekleta alang sa mga bisita sa park.</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>manakop og ligid</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>nga ang usa ka tawo naugtang sa usa ka sakyanan</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>['manakop', 'ligid']</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>"Manakop og ligid kaayo imong mga plano, walay klaro."</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>Si Juan ug iyang mga amigo nagsabot nga manakop og ligid alang sa ilang bag-ong negosyo nga vulcanizing shop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>manglutasay</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>usa ka manunulak sa mga bukog</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>['manglutasay']</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>Ang iyang kauban sa trabaho manglutasay sa mga kabataan.</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>Ang mga bata nagdula sa ilalom sa manglutasay aron magpa-uyog.</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>mag-ihaw og lata</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>sa pagluto sa mga pagkaon nga tinago</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>['mag-ihaw']</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>Si Juan pirmi lang mag-ihaw og lata sa boarding house.</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>Gikuha ni Pedro ang kalaha aron mag-ihaw og lata sa ilang umahan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>buhat ang pasulti-on dili sulti ang pabuhaton</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>Maglakaw sa paghisgot</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>['buhat', 'pasulti-on', 'sulti', 'pabuhaton']</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>Si Pedro nagpakita nga maayo siya sa trabaho, buhat ang pasulti-on dili sulti ang pabuhaton.</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>Gisuwayan ni Juan nga i-assemble ang kabayo-kabayo nga laruan gamit ang manual, buhat ang pasulti-on dili sulti ang pabuhaton.</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>bisan ang kabaw nga naay upat ka tiil masipyat</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>kitang tanan magkamali</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>['naay', 'masipyat']</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>Si Ana nakasala sa iyang trabaho, bisan ang kabaw nga naay upat ka tiil masipyat.</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>Naglakaw-lakaw ang kabaw sa uma, apan bisan ang kabaw nga naay upat ka tiil masipyat, natapilok siya.</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>makamala og sapa</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>ang usa ka tawo nga may dagkong tiil</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>['makamala']</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>Si Maria nagkatawa kay ang iyang igsuon makamala og sapa sa kadako sa tiil.</t>
-        </is>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>Ang mga trabahante nagkinahanglan og kahoy nga makamala og sapa aron makabalhin ang mga gamit ngadto sa pikas nga pampang.</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>pangatulig luwag</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>gigamit sa pag-undang sa usa ka tawo nga misquoted o misheard sa usa ka gisulti</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>Ang iyang giingon kay murag pangatulig luwag, dili ko kasabot.</t>
-        </is>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>Nag-uban mi sa kusina, ug gi-pangatulig luwag nako ang sinugba aron dili masunog.</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>halinon og aping</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>maayo kaayo nga hitsura</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>['halinon']</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>Ang mga artista kasagaran halinon og aping tungod sa ilang hitsura.</t>
-        </is>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>Ang iring namo halinon og aping tungod kay kanunay kini gihapuhap sa among pamilya.</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>abot na sa dukot</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>pag-iskrabe sa ubos sa bariles</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>['abot', 'dukot']</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>Ang iyang mga problema murag abot na sa dukot, grabe na kaayo.</t>
-        </is>
-      </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t>Nagkuha ko og sud-an sa kaldero, pero kinahanglan gyud nga aboton ang dukot aron mahurot ang kan-on.</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>kuyog baboy</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>usa ka tagalong</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>['kuyog']</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>Ang mga tawo nga kuyog baboy kasagaran magpalisod sa ilang mga kauban.</t>
-        </is>
-      </c>
-      <c r="E135" t="inlineStr">
-        <is>
-          <t>Miadto sila sa umahan uban sa ilang kuyog baboy nga gihiktan sa usa ka pisi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>pabuto</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>usa ka patok</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>['pabuto']</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr">
-        <is>
-          <t>Ang iyang surprise party kay murag pabuto nga naka-shock sa tanan.</t>
-        </is>
-      </c>
-      <c r="E136" t="inlineStr">
-        <is>
-          <t>Nagpalit mi ug daghang pabuto alang sa selebrasyon sa Bag-ong Tuig.</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>ang baka nisulod sa kulon</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>gigamit sa pagsulti sa usa nga siya usa ka bakak o ikaw mahimo sa pagsulti sa laing nagbuwa</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>['nisulod']</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>Ang ilang proyekto nga walay direksyon mura'g baka nga nisulod sa kulon.</t>
-        </is>
-      </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>Ang baka sa among uma nisulod sa dakong kulon sa kusina.</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>gidaman</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>sa pag-aturog o pag-aturog</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>['gidaman']</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>"Gidaman na ba ka? Daghan kaayo kag opinion."</t>
-        </is>
-      </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>Pagka-buntag, iyang mama miingon nga kagabii, gidaman diay siya ug naglakaw-lakaw sa sulod sa kwarto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>hinaw</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>sa paghunaw sa kamot sa usa o sa uban</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>['hinaw']</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>Si Pedro naghinaw sa iyang responsibilidad pagkahuman sa proyekto.</t>
-        </is>
-      </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>Si Maria naghinaw sa iyang mga kamot human mokaon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>bahong biyuda</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>adunay kusog nga baho nga musky o balsam</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>['bahong', 'biyuda']</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>Si Pedro bahong biyuda kay bisan unsaon ug ligo, dili mawala ang baho.</t>
-        </is>
-      </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>Ang silingan nagreklamo tungod kay ang tambong nga pagkahuman sa lamay sa hintungdan nga bahong biyuda pa gihapon hangtod karon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>baba sa atay</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>ang diaphragm</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>['baba']</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>Ang pag-amping sa baba sa atay usa ka importante nga parte sa pag-atiman sa lawas.</t>
-        </is>
-      </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>Gisuwayan ni Pedro pagkat-on ang posisyon sa baba sa atay sa klase sa anatomiya.</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>babayeng ikogan</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>transgender</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>['ikogan']</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>Si Pedro kay permi magbuang sa mga babayeng ikogan.</t>
-        </is>
-      </c>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>Ang mga sinuwaki nangga atong nakita kay babayeng ikogan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>ander de bunal</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>gi-squeeze</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>['bunal']</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>Si Pedro kay ander de bunal, kay pirmi lang musunod sa iyang asawa bisan unsa pa.</t>
-        </is>
-      </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>Ang bata nakuyawan pagkahuman nga ander de bunal siya sa iyang amahan tungod sa iyang pagkabadlong.</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>gwapa kon magtalikod</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>nindot nga tan-awon gikan sa likod</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>['magtalikod']</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>Si Maria pirmi lang ginatawgon nga gwapa kon magtalikod sa iyang mga amigo.</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>Pag-gawas ni Ana sa kwarto, giingnan siya sa iyang igsoong nga gwapa kon magtalikod kay nindot ang pagkasul-ot sa iyang sanina.</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>abot sa pikas bukid</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>usa ka tawo nga naghisgot nga makusog</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>['abot']</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>Ang iyang reklamo abot sa pikas bukid, grabe kaayo ug kasaba.</t>
-        </is>
-      </c>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>Migawas si Ana kada buntag aron mananom, ug dal-on niya ang iyang mga produkto abot sa pikas bukid alang sa pagbaligya.</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>kapugngan pa ang baha, dili ang biga</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>dili mapugngan</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>Ang iyang determinasyon dili mapugngan, kapugngan pa ang baha, dili ang biga.</t>
-        </is>
-      </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>Nagbungkag ang dakong kusog sa biga sa panagdait sa baryo, kapugngan pa ang baha, dili ang biga nga nagdala og kagubot sa mga tawo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>ul-ol</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>sa pag- masturba Mga sinonim: batil</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>['ul-ol']</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>Ang mga ul-ol nga tawo kasagaran dili makuha ang tinuod nga punto.</t>
-        </is>
-      </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>Naghilum siya sa kwarto ug nag-ul-ol sa dihang walay tawo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>gigukod sa plansa</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>ang usa ka tawo nga nagsul-ob ug mga sinina</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>['gigukod']</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>Ang iyang sinina pirmi lang gigukod sa plansa, maong bati tan-awon.</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>Ang bata mikatawa samtang gigukod sa plansa ang eroplano nga iyang gihimo gikan sa papel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>gwapa kon magtalikod</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>nindot nga tan-awon gikan sa likod</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>['magtalikod']</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>Ang mga tao nga gwapa kon magtalikod kasagaran maulaw kung mag-atubang.</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>"Si Ana gwapa kon magtalikod kay nindot ug straight ang iyang buhok."</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>dili tanang butang sili nga mohalang dayon</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>Dili tanan mahitabo sa usa ka higayon</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>['butang', 'mohalang']</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>Ang mga tawo nga dili tanang butang sili nga mohalang dayon kasagaran magmalampuson sa ilang mga plano.</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>Nagpalit siya og daghang klase sa sili sa merkado, pero nakadiskubre siya nga dili tanang butang sili nga mohalang dayon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>kusog mokaon og gasolina</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>gas-gussing</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>['mokaon']</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>Si Maria dili ganahan ug sakyanan nga kusog mokaon og gasolina kay mahal ang maintenance.</t>
-        </is>
-      </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>Ang bag-ong makina nga gisulayan nila sa laboratoryo kusog mokaon og gasolina sa paspas nga dagan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>mag-ugbok og mohon</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>sa pagpakigsekso</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>['mag-ugbok']</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>Ang magtiayon nagdecide nga mag-ugbok og mohon sa ilang honeymoon.</t>
-        </is>
-      </c>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>Ang mga trabahante mag-ugbok og mohon para sa bag-ong balay nga tukoron.</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>murag namiya og tai</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>Usa ka tawo nga mibiya sa dili-iasa nga walay iyang pulong</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>"Si Pedro murag namiya og tai, wala na gani nagpahibalo sa iyang mga kauban."</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>Pagkahuman kaon sa iyang pamahaw, si Jun-jun murag namiya og tai kay dali-dali nga midagan paingon sa kasilyas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>kulang sa tagad</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>kinaiya sa usa ka nagpangita ug atensyon</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>['tagad']</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>Si Maria kulang sa tagad, pirmi lang magbinuang aron makuha ang atensyon sa iyang mga kauban.</t>
-        </is>
-      </c>
-      <c r="E154" t="inlineStr">
-        <is>
-          <t>Ang balay ni Lolo ug Lola kulang sa tagad, mao nga hapit na mapapas ang ilang pintal ug nagkinahanglan na’g bag-ong kisame.</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>ang kalimot walay gahom</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>Ang pagkalimtan dili makahatag kanimo ug wala ka kaayohan</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>Ang mga estudyante nga malimot maglisod sa exam, ang kalimot walay gahom.</t>
-        </is>
-      </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t>Naa koy gipangita sa akong mga gamit, apan murag ang kalimot walay gahom, kay di man gihapon nako makita.</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>kuskos balungos</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>pag-awhag</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>['kuskos']</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>Si Pedro pirmi lang kuskos balungos sa iyang trabaho.</t>
-        </is>
-      </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t>Nagkuhaan si Maria ug dali nga kuskos balungos aron limpyohan ang lamesa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>gidaman</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>sa pag-aturog o pag-aturog</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>['gidaman']</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>"Kung mangutana ka og ing-ana, murag gidaman ka."</t>
-        </is>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>Pagmata nako sa buntag, nakita nako ang akong igsoon nga gidaman ug naglakaw-lakaw sa sala.</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>basa og baba</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>mabangis</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>['baba']</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>Si Juan basa og baba ug permi magdala ug kasaba sa opisina.</t>
-        </is>
-      </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t>Nagbasa og baba si Maria samtang nagbasa sa iyang paborito nga libro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>bibingkang liki</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>ang mga genital sa babaye</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>['liki']</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t>Ang bibingkang liki kay uso kaayo sa mga binuang ug katawa sa mga barkada.</t>
-        </is>
-      </c>
-      <c r="E159" t="inlineStr">
-        <is>
-          <t>Gipalit nako ang bibingkang liki sa merkado kay paborito gyud ni nako nga pagkaon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>magtumba og baka</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>sa pag-ihaw sa usa ka vaca</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>['magtumba']</t>
-        </is>
-      </c>
-      <c r="D160" t="inlineStr">
-        <is>
-          <t>Ang ilang pamilya magtumba og baka kung naa’y dako nga celebration.</t>
-        </is>
-      </c>
-      <c r="E160" t="inlineStr">
-        <is>
-          <t>Ang manggugubat magtumba og baka para sa karne nga ilang ipamaligya sa merkado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>walay mahay nga gauna</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>Ang nahimo dili mahimong malikayan</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>['mahay']</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>Si Pedro nakasabot nga walay mahay nga gauna, mao nga nagmatngon siya sa iyang mga desisyon.</t>
-        </is>
-      </c>
-      <c r="E161" t="inlineStr">
-        <is>
-          <t>Nagbasa si Ana ug libro ug nakahuna-huna, "Walay mahay nga gauna," samtang nagtan-aw siya sa mga mahay sa mga bakante nga panid sa sinugdanan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>manira sa dalan</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>aron magpabilin nga magmata hangtod sa gabii</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>"Si Ana, sige lang manira sa dalan walay klaro."</t>
-        </is>
-      </c>
-      <c r="E162" t="inlineStr">
-        <is>
-          <t>"Ang mga estudyante manira sa dalan aron dili maligsan samtang nagduwa."</t>
+          <t>"Nakit-an nako si Lito nga nagkuha og sungkod aron magtuslok baki sa daplin sa sapa."</t>
         </is>
       </c>
     </row>

</xml_diff>